<commit_message>
B2B approfondi : fil de discussion, commande, confirmation, livraison, reception, notifications
Une page par negociation, les gestes de chaque partie sous sa propre
habilitation. Demande de prix ou commande directe ; contre-propositions ;
le fournisseur confirme selon son stock (son BC nait), livre et facture par
la porte habituelle ; le client receptionne (sa facture d'achat nait).
Courriel a l'autre partie et pastilles non lu.

Corrige : b2b_negotiation_id absent des champs remplissables d'Achat et de
Vente (aucune piece n'etait rattachee) ; BC d'un vendeur pour un client
inscrit transmis a l'envers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -905,7 +905,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>9. B2B APPROFONDI — validé le 14/10, à programmer</t>
+          <t>9. B2B APPROFONDI — validé et livré le 14/10 (lot 75)</t>
         </is>
       </c>
       <c r="B13" s="15" t="n">
@@ -915,10 +915,10 @@
         <v>4</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>0</v>
@@ -926,9 +926,9 @@
       <c r="G13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -942,10 +942,10 @@
         <v>34</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>3</v>
@@ -2286,7 +2286,7 @@
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
-          <t>9. B2B APPROFONDI — validé le 14/10, à programmer</t>
+          <t>9. B2B APPROFONDI — validé et livré le 14/10 (lot 75)</t>
         </is>
       </c>
       <c r="B51" s="21" t="n"/>
@@ -2315,18 +2315,20 @@
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
-          <t>Messages horodatés des deux côtés, contre-proposition ligne à ligne, badge, courriel à l'autre partie.</t>
-        </is>
-      </c>
-      <c r="E52" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Une page par négociation : étapes, lignes, échanges en bulles ; contre-proposition ligne à ligne (lot 75).</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F52" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G52" s="22" t="n"/>
+      <c r="G52" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H52" s="15" t="inlineStr">
         <is>
           <t>Jour 1</t>
@@ -2351,18 +2353,20 @@
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>« Commander » après une demande de prix ou directement (accordé le 14/10) ; le fournisseur confirme selon son stock → « Confirmé — en attente de livraison ». Corrige l'inversion client / fournisseur et les références manquantes.</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>« Commander » après une demande de prix ou directement (accordé le 14/10) ; le fournisseur confirme selon son stock → « Confirmé — en attente de livraison ». Inversion client / fournisseur corrigée ; pièces enfin rattachées à leur négociation (lot 75).</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F53" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G53" s="22" t="n"/>
+      <c r="G53" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H53" s="15" t="inlineStr">
         <is>
           <t>Jour 1</t>
@@ -2387,18 +2391,20 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>BL, facture certifiée du fournisseur ; le client réceptionne → stock et facture d'achat informative.</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Facture par la porte habituelle (FNE comprise) ; le client réceptionne → stock et facture d'achat, déclarée par le fournisseur si certifiée (lot 75).</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F54" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G54" s="22" t="n"/>
+      <c r="G54" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
           <t>Jour 1</t>
@@ -2423,18 +2429,20 @@
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>Courriel et compteur au menu à chaque changement d'état.</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Courriel aux administrateurs de l'autre partie ; pastille « non lu » au menu et dans les listes (lot 75).</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F55" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G55" s="22" t="n"/>
+      <c r="G55" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H55" s="15" t="inlineStr">
         <is>
           <t>Jour 1</t>

</xml_diff>

<commit_message>
Plans : retours du 15/10 (lots 76 à 78) et les quatre modes d'usage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -933,24 +933,54 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>10. RETOURS DU 15/10 — inscription, fiscalité, achat, pas à pas</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>6/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="E14" s="10" t="n">
+      <c r="C15" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="E15" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" s="10" t="n">
+      <c r="F15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -966,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2449,8 +2479,320 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1"/>
-    <row r="64" ht="20" customHeight="1"/>
+    <row r="57">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>10. RETOURS DU 15/10 — inscription, fiscalité, achat, pas à pas</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="n"/>
+      <c r="C57" s="21" t="n"/>
+      <c r="D57" s="21" t="n"/>
+      <c r="E57" s="21" t="n"/>
+      <c r="F57" s="21" t="n"/>
+      <c r="G57" s="21" t="n"/>
+      <c r="H57" s="21" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Inscription</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>URGENT — l'étape 3 facultative exigeait l'accès FNE</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>Un NCC incomplet refusait la création de l'entreprise. Il est désormais écarté et signalé ; l'entreprise est créée (lot 76).</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G58" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>Saisie</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Vendre, acheter, facturer sans information fiscale</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>Ventes et achats ne sont plus retenus que faute de point de vente ; NCC, RCCM, régime, domaine n'y sont plus exigés (lot 76).</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F59" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G59" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H59" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Normalisation</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Le blocage à la normalisation, avec Remplir / Fermer</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>Normaliser sans NCC, régime, point de vente ou accès FNE ouvre « Informations fiscales non renseignées » avec la liste, « Remplir » et « Fermer » ; l'automatique laisse la pièce à normaliser sans rejet (lot 76).</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G60" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H60" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Factures</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Le NCC posé plus tard paraît sur les factures</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>Les impressions lisent le NCC au moment d'imprimer : rien à changer, épreuve ajoutée (lot 76).</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G61" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H61" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Achats</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Aucun moyen de paiement pour une DP ou un BC</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>Le règlement restait affiché après « Facture physique » puis DP/BC, et le serveur enregistrait « Caisse ». Corrigé des deux côtés (lot 77).</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F62" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G62" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H62" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Achats</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>La page achat nécessite-t-elle une refonte ?</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>Cohérente une fois le défaut levé. Une version « pas à pas » comme la vente est possible : à décider.</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G63" s="22" t="n"/>
+      <c r="H63" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Vente pas à pas</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>10.7</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Voir et régler TVA, remise par ligne (inspiration Odoo)</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>Chaque ligne choisie s'ouvre en boîte : quantité, unité, remise, code TVA, total ; la TVA de la fiche se lit avant l'ajout ; lignes libres visibles (lot 78).</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F64" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G64" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H64" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>Modes d'usage</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>10.8</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Les quatre modes (normaliser ou non × écritures ou non)</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Pris en charge ; les écritures restent tenues en arrière-plan quand la comptabilité est fermée (décision du lot 5). Les couper tout à fait : à décider.</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F65" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G65" s="22" t="n"/>
+      <c r="H65" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
     <row r="72" ht="20" customHeight="1"/>
     <row r="78" ht="20" customHeight="1"/>
     <row r="84" ht="20" customHeight="1"/>
@@ -2465,13 +2807,14 @@
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H56"/>
-  <mergeCells count="9">
+  <autoFilter ref="A4:H66"/>
+  <mergeCells count="10">
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A57:H57"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A32:H32"/>

</xml_diff>

<commit_message>
Plans : retours du 15/10 au soir (lots 79 à 81)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -963,24 +963,54 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>11. RETOURS DU 15/10 (soir) — pannes, superadmin, abonnements</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>67</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>8/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>37</v>
-      </c>
-      <c r="E15" s="10" t="n">
+      <c r="C16" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="E16" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="G15" s="10" t="n">
+      <c r="F16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -996,7 +1026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2793,7 +2823,360 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="20" customHeight="1"/>
+    <row r="67">
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>11. RETOURS DU 15/10 (soir) — pannes, superadmin, abonnements</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="n"/>
+      <c r="C67" s="21" t="n"/>
+      <c r="D67" s="21" t="n"/>
+      <c r="E67" s="21" t="n"/>
+      <c r="F67" s="21" t="n"/>
+      <c r="G67" s="21" t="n"/>
+      <c r="H67" s="21" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Pannes</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Page de maintenance au lieu de l'erreur</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>« En maintenance, résolu dans un instant », la référence et les contacts de l'assistance saisis par le superadmin ; plus aucun détail technique à l'écran (lot 79).</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F68" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G68" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H68" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Pannes</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Registre des pannes au superadmin</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>Code et adresse par ligne, l'erreur au clic ; « Corrigée » ou fermeture d'elle-même quand le fichier fautif a changé ; revient si elle se reproduit (lot 79).</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F69" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G69" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H69" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Secteurs : le même parcours, avec « Suivant »</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>« Suivant » crée l'entreprise et déroule pour elle le parcours de configuration complet ; bouton « Parcours » dans la liste (lot 80).</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G70" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Quota par défaut 3, modules retirés</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>3 points de vente pour les futures entreprises, les anciennes gardent les leurs ; tableau des modules retiré (lot 80).</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F71" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G71" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Mot de passe : « Voir » et barre de précision</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>Un clic ouvre les deux champs ; règles cochées en direct et jauge de solidité (lot 80).</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F72" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G72" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Bloc FNE mal présenté, choix impossible à retirer</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>Mise en forme propre au bloc ; un second clic retire le choix (lot 80).</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F73" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G73" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Aligner le superadmin sur les décisions</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>Forme juridique et compte contribuable retirés, doublons fiscaux supprimés, donnée fiscale mal formée écartée et non refusée, domaine non exigé à la modification (lot 80).</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F74" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G74" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Solo, Business, Premium, Sur mesure, Pass cadeau</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>Cartes après l'inscription et en vitrine ; limites de points de vente et d'utilisateurs appliquées ; le superadmin les relève sans changer d'offre (lot 81).</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F75" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G75" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>11.9</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Paiement et fin du pass cadeau</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>Aucun paiement en ligne : une offre payante reste « à régler ». À la fin du pass, un bandeau seulement. Bloquer ? Encaisser comment ?</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G76" s="22" t="n"/>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
     <row r="78" ht="20" customHeight="1"/>
     <row r="84" ht="20" customHeight="1"/>
     <row r="89" ht="20" customHeight="1"/>
@@ -2807,8 +3190,9 @@
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H66"/>
-  <mergeCells count="10">
+  <autoFilter ref="A4:H77"/>
+  <mergeCells count="11">
+    <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A46:H46"/>

</xml_diff>

<commit_message>
Plans : retours du 15/10 dans la nuit (lots 82 et 83)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -993,24 +993,54 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>12. RETOURS DU 15/10 (nuit) — habilitations, facturation, échéance</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>78</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
-        <v>51</v>
-      </c>
-      <c r="D16" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="E16" s="10" t="n">
+      <c r="C17" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="E17" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="10" t="n">
+      <c r="F17" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1026,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3159,12 +3189,12 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Aucun paiement en ligne : une offre payante reste « à régler ». À la fin du pass, un bandeau seulement. Bloquer ? Encaisser comment ?</t>
+          <t>Tranché le 15/10 : à l'échéance, l'espace est bloqué (voir 12.3). L'API de paiement arrive : en attendant, DC-Knowing confirme le règlement.</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
         <is>
-          <t>À trancher</t>
+          <t>Attendu</t>
         </is>
       </c>
       <c r="F76" s="22" t="n">
@@ -3177,7 +3207,208 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="20" customHeight="1"/>
+    <row r="78">
+      <c r="A78" s="23" t="inlineStr">
+        <is>
+          <t>12. RETOURS DU 15/10 (nuit) — habilitations, facturation, échéance</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="n"/>
+      <c r="C78" s="21" t="n"/>
+      <c r="D78" s="21" t="n"/>
+      <c r="E78" s="21" t="n"/>
+      <c r="F78" s="21" t="n"/>
+      <c r="G78" s="21" t="n"/>
+      <c r="H78" s="21" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>URGENT — mettre à jour les habilitations</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>Produits et Tiers manquaient à la liste ; sept écrans prennent leur droit (livraisons, B2B, Fiscalité &amp; DGI, stickers, consignations, immobilisations, paramètres) ; personne ne perd un écran (lot 82).</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F79" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G79" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Paramètres</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Section Facturation avec cartes</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>Offre, échéance, consommation ; cartes avec avantages : renouveler, passer à une offre supérieure (lot 83).</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F80" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G80" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H80" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Bloquer l'accès à l'échéance</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>Espace visible mais inerte, fenêtre « Abonnement à terme » avec Continuer vers la facturation ; le serveur refuse toute action (lot 83).</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F81" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G81" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Paramétrage</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>12.4</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Métier Poissonnerie</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>Nouveau métier du parcours (Commerce) : familles et 22 articles (lot 83).</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F82" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G82" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>API de paiement</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>À brancher dès qu'elle est disponible : elle repoussera l'échéance à la place de DC-Knowing.</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Attendu</t>
+        </is>
+      </c>
+      <c r="F83" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G83" s="22" t="n"/>
+      <c r="H83" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
     <row r="84" ht="20" customHeight="1"/>
     <row r="89" ht="20" customHeight="1"/>
     <row r="94" ht="20" customHeight="1"/>
@@ -3190,10 +3421,11 @@
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H77"/>
-  <mergeCells count="11">
+  <autoFilter ref="A4:H84"/>
+  <mergeCells count="12">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A78:H78"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A12:H12"/>

</xml_diff>

<commit_message>
Plans : lots 84 et 85
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -975,20 +975,20 @@
         <v>9</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>8/9</t>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1002,10 +1002,10 @@
         <v>78</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>0</v>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>6/7</t>
         </is>
       </c>
     </row>
@@ -1029,16 +1029,16 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G17" s="10" t="n">
         <v>0</v>
@@ -1056,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3184,23 +3184,25 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Paiement et fin du pass cadeau</t>
+          <t>Fin du pass cadeau</t>
         </is>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Tranché le 15/10 : à l'échéance, l'espace est bloqué (voir 12.3). L'API de paiement arrive : en attendant, DC-Knowing confirme le règlement.</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>Attendu</t>
+          <t>Tranché le 15/10 : oui, l'accès est bloqué à la fin des 7 jours (lots 83 et 85).</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F76" s="22" t="n">
         <v>46310</v>
       </c>
-      <c r="G76" s="22" t="n"/>
+      <c r="G76" s="22" t="n">
+        <v>46310</v>
+      </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
           <t>Jour 2</t>
@@ -3376,40 +3378,115 @@
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
         <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>12.6</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>« Suivant » du domaine bloquait toute la page</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>Le parcours se déroule dans la section (domaine, métiers, modules, rayons) sans soumettre ; appliqué à la création, puis prix et stock (lot 85).</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F83" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G83" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H83" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>12.7</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Erreur 500 à la suppression d'une entreprise</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>Suppression en une transaction, en suivant les dépendances ; « eve disagn » avait perdu ses utilisateurs : relancer la suppression après déploiement (lot 84).</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F84" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G84" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H84" s="15" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
           <t>Abonnements</t>
         </is>
       </c>
-      <c r="B83" s="15" t="inlineStr">
+      <c r="B85" s="15" t="inlineStr">
         <is>
           <t>12.5</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>API de paiement</t>
         </is>
       </c>
-      <c r="D83" s="14" t="inlineStr">
+      <c r="D85" s="14" t="inlineStr">
         <is>
           <t>À brancher dès qu'elle est disponible : elle repoussera l'échéance à la place de DC-Knowing.</t>
         </is>
       </c>
-      <c r="E83" s="18" t="inlineStr">
+      <c r="E85" s="18" t="inlineStr">
         <is>
           <t>Attendu</t>
         </is>
       </c>
-      <c r="F83" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G83" s="22" t="n"/>
-      <c r="H83" s="15" t="inlineStr">
+      <c r="F85" s="22" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G85" s="22" t="n"/>
+      <c r="H85" s="15" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="20" customHeight="1"/>
     <row r="89" ht="20" customHeight="1"/>
     <row r="94" ht="20" customHeight="1"/>
     <row r="100" ht="20" customHeight="1"/>
@@ -3421,7 +3498,7 @@
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H84"/>
+  <autoFilter ref="A4:H86"/>
   <mergeCells count="12">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>

</xml_diff>

<commit_message>
Plans et passation : retours du 16/10/2026 (lots 86 à 94)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -165,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -228,6 +229,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -593,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -836,7 +838,7 @@
       <c r="G10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
@@ -896,7 +898,7 @@
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
@@ -956,7 +958,7 @@
       <c r="G14" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>6/8</t>
         </is>
@@ -1002,10 +1004,10 @@
         <v>78</v>
       </c>
       <c r="C16" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="15" t="n">
         <v>7</v>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>6</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>0</v>
@@ -1016,31 +1018,61 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>6/7</t>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>7/8</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>13. RETOURS DU 16/10 — immobilisations, annulation, paiements, liaisons, sécurité</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>88</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>13/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n">
-        <v>58</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>52</v>
-      </c>
-      <c r="E17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="10" t="n">
+      <c r="C18" t="n">
+        <v>74</v>
+      </c>
+      <c r="D18" t="n">
+        <v>66</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G17" s="10" t="n">
+      <c r="G18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1056,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1126,204 +1158,197 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>1. SÉCURITÉ ET COURRIELS — le mot de passe oublié</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
-      <c r="F5" s="21" t="n"/>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Mot de passe oublié</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Le lien de réinitialisation ne s'affiche plus à l'écran</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Faille : le lien s'affichait à quiconque tapait une adresse, en production. Il ne part plus que par courriel ; même réponse que l'adresse existe ou non ; jeton vérifié avant le formulaire (lot 64).</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G6" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Courriels</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Le courriel part réellement</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Transport « log » par défaut : rien ne partait. EnvoiCourriel dit l'échec ; commande selflow:verifier-courriel. Vérifié en production le 14/10 (SMTP mail.dc-knowing.com, message d'essai remis).</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G7" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Courriels</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Avis d'ouverture de compte</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Inscription, employé (écran et API), responsable créé par le superadmin, admin interne : le titulaire est prévenu, sans mot de passe (lot 64).</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F8" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G8" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Mot de passe oublié</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Page « 429 Too Many Requests »</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Borne comptée par adresse saisie (3 / 15 min) et non par IP de bureau ; page lisible avec message ; envoi du nouveau mot de passe borné à part (lot 71).</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F9" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H9" s="15" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Mot de passe</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Préciser les caractères à saisir</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Liste cochée en direct sous le champ : 8 caractères (obligatoire), majuscule, minuscule, chiffre, caractère spécial (lot 71).</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F10" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G10" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
@@ -1331,918 +1356,875 @@
     </row>
     <row r="11" ht="20" customHeight="1"/>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2. VENTES — la caisse et la vente pas à pas</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="21" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Nouvelle vente</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>La facture « ne passe pas », sans message</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Refus de stock et de lot périmé perdus sous la clé error : affichés ; refus sous verrou rendus en message (lot 65).</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F13" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G13" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Nouvelle vente</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Message de confirmation de 3 secondes</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>« Facture VTE-… enregistrée », 3 s ; panier vidé après la vente (lot 65).</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F14" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G14" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Nouvelle vente</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Nouvelle présentation : la vente pas à pas</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Bascule Caisse / Pas à pas : articles, client et document, règlement, valider et facturer ; même formulaire, rien ne change côté FNE (lot 69).</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F15" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G15" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Nouvelle vente</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Refonte de l'étape 1 « Articles »</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Liste plein écran au lieu des tuiles : une ligne par article avec compteur − / + ; barre fixe en bas (articles, net à payer, suite) ; plus de panier latéral à cette étape (lot 74). À valider à l'usage.</t>
         </is>
       </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F16" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G16" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Nouvelle vente</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Catégorie sans nom dans les filtres</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Pastille vide pour les articles sans catégorie : « Sans catégorie » (lot 74).</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F17" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G17" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>3. ÉCRANS — ce que le retest a relevé</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="21" t="n"/>
-      <c r="F19" s="21" t="n"/>
-      <c r="G19" s="21" t="n"/>
-      <c r="H19" s="21" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Tableau de bord</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Retirer la fusée de la bannière</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Retirée (lot 65).</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F20" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G20" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Profil</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Image cassée sans photo</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Initiales par défaut ; photo Google refusée par la politique de sécurité, fichier disparu, initiale accentuée : tous retombent sur les initiales (lot 65).</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F21" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G21" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Paramètres</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Domaine : aller à l'étape suivante d'un clic</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Le clic mène à l'étape 2 (lot 65). Défaut du soir : après « Retour » du navigateur, le clic restait sans effet (page restaurée avec son drapeau « envoyé ») — corrigé (lot 74).</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G22" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>La recherche ne voit que la page affichée</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Recherche serveur sur tout le catalogue, pagination qui garde les filtres (lot 65).</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F23" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G23" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Recherches</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>La page se recharge à chaque caractère</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Dix écrans : la recherche part par Entrée ou par le bouton (lot 71).</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F24" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G24" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>4. ACHATS — le cycle d'achat</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="21" t="n"/>
-      <c r="G26" s="21" t="n"/>
-      <c r="H26" s="21" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Bon d'achat</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Un seul bouton selon l'étape</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Demande de prix → Confirmer la commande ; commande → Bon de réception et Valider &amp; Facturer (lot 66).</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F27" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G27" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Liste des achats</t>
         </is>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Actions sur les demandes et les commandes</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Confirmer la commande, Facturer ; facture informative signalée (lot 66).</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F28" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G28" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H28" s="15" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Facturation</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Facture déclarée par le fournisseur</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Question à la facturation : oui → saisie informative, la facture reçue de la DGI porte l'écriture ; non → écriture comme avant (lot 66).</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F29" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G29" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Achat B2B écrit « Bon de Commande »</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>C majuscule : échappait aux contrôles ; corrigé, données reprises par migration (lot 66).</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F30" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G30" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H30" s="15" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>5. COMPTABILITÉ — avoirs et plan comptable</t>
         </is>
       </c>
-      <c r="B32" s="21" t="n"/>
-      <c r="C32" s="21" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="21" t="n"/>
-      <c r="F32" s="21" t="n"/>
-      <c r="G32" s="21" t="n"/>
-      <c r="H32" s="21" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Avoirs</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>L'avoir, écriture d'origine en négatif</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Taxes parafiscales contre-passées ; remboursement en espèces écrit (411 / caisse) ; retour au coût de sortie (lot 67).</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F33" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G33" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H33" s="15" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Avoirs</t>
         </is>
       </c>
-      <c r="B34" s="15" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Le timbre d'une facture annulée</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Tranché le 14/10 : non remboursé, il reste dû à l'État (la plateforme ne le porte sur aucun avoir).</t>
         </is>
       </c>
-      <c r="E34" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F34" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G34" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H34" s="15" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Plan comptable</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Modifier et supprimer les comptes créés</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Seulement les comptes créés par l'entreprise ; un compte employé garde son numéro et ne se supprime pas (lot 72).</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F35" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G35" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H35" s="15" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>6. FISCALITÉ ET STICKERS</t>
         </is>
       </c>
-      <c r="B37" s="21" t="n"/>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="21" t="n"/>
-      <c r="E37" s="21" t="n"/>
-      <c r="F37" s="21" t="n"/>
-      <c r="G37" s="21" t="n"/>
-      <c r="H37" s="21" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Stickers</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>L'achat des stickers, confié à DC-Knowing</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Demande gardée, courriel à DC-Knowing et accusé au demandeur, page superadmin avec statut (lot 68).</t>
         </is>
       </c>
-      <c r="E38" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F38" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G38" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H38" s="15" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Gestion FNE</t>
         </is>
       </c>
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Les données du timbre sont-elles récupérées ?</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Oui, mais seulement par les réponses de certification : la page le dit et compte les factures non normalisées ; proformas « non transmis » (lot 72).</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F39" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G39" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H39" s="15" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Fiscalité &amp; DGI</t>
         </is>
       </c>
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Revoir l'affichage des sous-modules</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Le défaut d'affichage n'est pas identifié : préciser l'écran et ce qui ne va pas.</t>
         </is>
       </c>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F40" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G40" s="22" t="n"/>
-      <c r="H40" s="15" t="inlineStr">
+      <c r="F40" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>7. ARTICLES ET STOCK</t>
         </is>
       </c>
-      <c r="B42" s="21" t="n"/>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="21" t="n"/>
-      <c r="F42" s="21" t="n"/>
-      <c r="G42" s="21" t="n"/>
-      <c r="H42" s="21" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Fiche article</t>
         </is>
       </c>
-      <c r="B43" s="15" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Erreur 500 en ligne à la création d'un article</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>« Nouvelle catégorie » sans nom : la chaîne partait en base, MySQL la refusait. Catégorie et sous-catégorie validées ; celle d'une autre entreprise refusée (lot 71).</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F43" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G43" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H43" s="15" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G43" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Inventaire</t>
         </is>
       </c>
-      <c r="B44" s="15" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Import refusé à cause de la référence</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Modèle rempli des articles de l'entreprise ; référence sans casse, repli sur la désignation ; lignes vides ignorées ; « 0 importée » n'est plus vert (lot 71).</t>
         </is>
       </c>
-      <c r="E44" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F44" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G44" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H44" s="15" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G44" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
@@ -2250,1246 +2232,1812 @@
     </row>
     <row r="45" ht="20" customHeight="1"/>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>8. PAGE D'ACCUEIL</t>
         </is>
       </c>
-      <c r="B46" s="21" t="n"/>
-      <c r="C46" s="21" t="n"/>
-      <c r="D46" s="21" t="n"/>
-      <c r="E46" s="21" t="n"/>
-      <c r="F46" s="21" t="n"/>
-      <c r="G46" s="21" t="n"/>
-      <c r="H46" s="21" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Vitrine</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>8.1</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Le menu n'est pas bon</t>
         </is>
       </c>
-      <c r="D47" s="14" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Entrées courtes sur une ligne, menu « burger » sous 1 100 px ; contraste du haut de page (lot 73).</t>
         </is>
       </c>
-      <c r="E47" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F47" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G47" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H47" s="15" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Vitrine</t>
         </is>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>8.2</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Liens et descriptions des applications</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Selflow et Comptaflow mènent à leur site (lot 73). Textes et adresses de RHFlow, LegalFlow, Agent-AI, CGA-Connect : attendus du propriétaire.</t>
         </is>
       </c>
-      <c r="E48" s="18" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Attendu</t>
         </is>
       </c>
-      <c r="F48" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G48" s="22" t="n"/>
-      <c r="H48" s="15" t="inlineStr">
+      <c r="F48" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="14" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Vitrine</t>
         </is>
       </c>
-      <c r="B49" s="15" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>8.3</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>La section « Le cabinet » est-elle nécessaire ?</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Une phrase et une fiche : la compléter (présentation, photo) ou la masquer depuis Superadmin › Vitrine.</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F49" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G49" s="22" t="n"/>
-      <c r="H49" s="15" t="inlineStr">
+      <c r="F49" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="23" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>9. B2B APPROFONDI — validé et livré le 14/10 (lot 75)</t>
         </is>
       </c>
-      <c r="B51" s="21" t="n"/>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="21" t="n"/>
-      <c r="E51" s="21" t="n"/>
-      <c r="F51" s="21" t="n"/>
-      <c r="G51" s="21" t="n"/>
-      <c r="H51" s="21" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>70a — Fil de discussion</t>
         </is>
       </c>
-      <c r="D52" s="14" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Une page par négociation : étapes, lignes, échanges en bulles ; contre-proposition ligne à ligne (lot 75).</t>
         </is>
       </c>
-      <c r="E52" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F52" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G52" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H52" s="15" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G52" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="B53" s="15" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>70b — Commander et confirmer</t>
         </is>
       </c>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>« Commander » après une demande de prix ou directement (accordé le 14/10) ; le fournisseur confirme selon son stock → « Confirmé — en attente de livraison ». Inversion client / fournisseur corrigée ; pièces enfin rattachées à leur négociation (lot 75).</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F53" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G53" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H53" s="15" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G53" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="B54" s="15" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>9.3</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>70c — Livrer, facturer, réceptionner</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Facture par la porte habituelle (FNE comprise) ; le client réceptionne → stock et facture d'achat, déclarée par le fournisseur si certifiée (lot 75).</t>
         </is>
       </c>
-      <c r="E54" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F54" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G54" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H54" s="15" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G54" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="B55" s="15" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>9.4</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>70d — Notifications</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Courriel aux administrateurs de l'autre partie ; pastille « non lu » au menu et dans les listes (lot 75).</t>
         </is>
       </c>
-      <c r="E55" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F55" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G55" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H55" s="15" t="inlineStr">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H55" t="inlineStr">
         <is>
           <t>Jour 1</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="23" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>10. RETOURS DU 15/10 — inscription, fiscalité, achat, pas à pas</t>
         </is>
       </c>
-      <c r="B57" s="21" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
-      <c r="E57" s="21" t="n"/>
-      <c r="F57" s="21" t="n"/>
-      <c r="G57" s="21" t="n"/>
-      <c r="H57" s="21" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Inscription</t>
         </is>
       </c>
-      <c r="B58" s="15" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>10.1</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>URGENT — l'étape 3 facultative exigeait l'accès FNE</t>
         </is>
       </c>
-      <c r="D58" s="14" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Un NCC incomplet refusait la création de l'entreprise. Il est désormais écarté et signalé ; l'entreprise est créée (lot 76).</t>
         </is>
       </c>
-      <c r="E58" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F58" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G58" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H58" s="15" t="inlineStr">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G58" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H58" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="14" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Saisie</t>
         </is>
       </c>
-      <c r="B59" s="15" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>10.2</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Vendre, acheter, facturer sans information fiscale</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Ventes et achats ne sont plus retenus que faute de point de vente ; NCC, RCCM, régime, domaine n'y sont plus exigés (lot 76).</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F59" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G59" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H59" s="15" t="inlineStr">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F59" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G59" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H59" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="14" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Normalisation</t>
         </is>
       </c>
-      <c r="B60" s="15" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>10.3</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Le blocage à la normalisation, avec Remplir / Fermer</t>
         </is>
       </c>
-      <c r="D60" s="14" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>Normaliser sans NCC, régime, point de vente ou accès FNE ouvre « Informations fiscales non renseignées » avec la liste, « Remplir » et « Fermer » ; l'automatique laisse la pièce à normaliser sans rejet (lot 76).</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F60" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G60" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H60" s="15" t="inlineStr">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F60" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G60" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H60" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Factures</t>
         </is>
       </c>
-      <c r="B61" s="15" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Le NCC posé plus tard paraît sur les factures</t>
         </is>
       </c>
-      <c r="D61" s="14" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>Les impressions lisent le NCC au moment d'imprimer : rien à changer, épreuve ajoutée (lot 76).</t>
         </is>
       </c>
-      <c r="E61" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F61" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G61" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H61" s="15" t="inlineStr">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F61" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G61" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H61" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>Achats</t>
         </is>
       </c>
-      <c r="B62" s="15" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>10.5</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Aucun moyen de paiement pour une DP ou un BC</t>
         </is>
       </c>
-      <c r="D62" s="14" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>Le règlement restait affiché après « Facture physique » puis DP/BC, et le serveur enregistrait « Caisse ». Corrigé des deux côtés (lot 77).</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F62" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G62" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H62" s="15" t="inlineStr">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F62" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G62" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Achats</t>
         </is>
       </c>
-      <c r="B63" s="15" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>10.6</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>La page achat nécessite-t-elle une refonte ?</t>
         </is>
       </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Cohérente une fois le défaut levé. Une version « pas à pas » comme la vente est possible : à décider.</t>
         </is>
       </c>
-      <c r="E63" s="18" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F63" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G63" s="22" t="n"/>
-      <c r="H63" s="15" t="inlineStr">
+      <c r="F63" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H63" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Vente pas à pas</t>
         </is>
       </c>
-      <c r="B64" s="15" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>10.7</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>Voir et régler TVA, remise par ligne (inspiration Odoo)</t>
         </is>
       </c>
-      <c r="D64" s="14" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Chaque ligne choisie s'ouvre en boîte : quantité, unité, remise, code TVA, total ; la TVA de la fiche se lit avant l'ajout ; lignes libres visibles (lot 78).</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F64" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G64" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H64" s="15" t="inlineStr">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F64" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G64" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H64" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Modes d'usage</t>
         </is>
       </c>
-      <c r="B65" s="15" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>Les quatre modes (normaliser ou non × écritures ou non)</t>
         </is>
       </c>
-      <c r="D65" s="14" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Pris en charge ; les écritures restent tenues en arrière-plan quand la comptabilité est fermée (décision du lot 5). Les couper tout à fait : à décider.</t>
         </is>
       </c>
-      <c r="E65" s="18" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F65" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G65" s="22" t="n"/>
-      <c r="H65" s="15" t="inlineStr">
+      <c r="F65" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H65" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="23" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>11. RETOURS DU 15/10 (soir) — pannes, superadmin, abonnements</t>
         </is>
       </c>
-      <c r="B67" s="21" t="n"/>
-      <c r="C67" s="21" t="n"/>
-      <c r="D67" s="21" t="n"/>
-      <c r="E67" s="21" t="n"/>
-      <c r="F67" s="21" t="n"/>
-      <c r="G67" s="21" t="n"/>
-      <c r="H67" s="21" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="14" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>Pannes</t>
         </is>
       </c>
-      <c r="B68" s="15" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>11.1</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>Page de maintenance au lieu de l'erreur</t>
         </is>
       </c>
-      <c r="D68" s="14" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>« En maintenance, résolu dans un instant », la référence et les contacts de l'assistance saisis par le superadmin ; plus aucun détail technique à l'écran (lot 79).</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F68" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G68" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H68" s="15" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F68" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G68" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H68" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>Pannes</t>
         </is>
       </c>
-      <c r="B69" s="15" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>11.2</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Registre des pannes au superadmin</t>
         </is>
       </c>
-      <c r="D69" s="14" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>Code et adresse par ligne, l'erreur au clic ; « Corrigée » ou fermeture d'elle-même quand le fichier fautif a changé ; revient si elle se reproduit (lot 79).</t>
         </is>
       </c>
-      <c r="E69" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F69" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G69" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H69" s="15" t="inlineStr">
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F69" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G69" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H69" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B70" s="15" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>11.3</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Secteurs : le même parcours, avec « Suivant »</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>« Suivant » crée l'entreprise et déroule pour elle le parcours de configuration complet ; bouton « Parcours » dans la liste (lot 80).</t>
         </is>
       </c>
-      <c r="E70" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F70" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G70" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H70" s="15" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F70" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G70" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H70" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="14" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B71" s="15" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>11.4</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>Quota par défaut 3, modules retirés</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>3 points de vente pour les futures entreprises, les anciennes gardent les leurs ; tableau des modules retiré (lot 80).</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F71" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G71" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H71" s="15" t="inlineStr">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G71" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H71" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="14" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B72" s="15" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>11.5</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Mot de passe : « Voir » et barre de précision</t>
         </is>
       </c>
-      <c r="D72" s="14" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>Un clic ouvre les deux champs ; règles cochées en direct et jauge de solidité (lot 80).</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F72" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G72" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H72" s="15" t="inlineStr">
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F72" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G72" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H72" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="14" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B73" s="15" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>11.6</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Bloc FNE mal présenté, choix impossible à retirer</t>
         </is>
       </c>
-      <c r="D73" s="14" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Mise en forme propre au bloc ; un second clic retire le choix (lot 80).</t>
         </is>
       </c>
-      <c r="E73" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F73" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G73" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H73" s="15" t="inlineStr">
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F73" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G73" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H73" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B74" s="15" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>11.7</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Aligner le superadmin sur les décisions</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Forme juridique et compte contribuable retirés, doublons fiscaux supprimés, donnée fiscale mal formée écartée et non refusée, domaine non exigé à la modification (lot 80).</t>
         </is>
       </c>
-      <c r="E74" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F74" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G74" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H74" s="15" t="inlineStr">
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F74" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G74" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H74" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>Abonnements</t>
         </is>
       </c>
-      <c r="B75" s="15" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>11.8</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Solo, Business, Premium, Sur mesure, Pass cadeau</t>
         </is>
       </c>
-      <c r="D75" s="14" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>Cartes après l'inscription et en vitrine ; limites de points de vente et d'utilisateurs appliquées ; le superadmin les relève sans changer d'offre (lot 81).</t>
         </is>
       </c>
-      <c r="E75" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F75" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G75" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H75" s="15" t="inlineStr">
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F75" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G75" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H75" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>Abonnements</t>
         </is>
       </c>
-      <c r="B76" s="15" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>11.9</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>Fin du pass cadeau</t>
         </is>
       </c>
-      <c r="D76" s="14" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Tranché le 15/10 : oui, l'accès est bloqué à la fin des 7 jours (lots 83 et 85).</t>
         </is>
       </c>
-      <c r="E76" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F76" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G76" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H76" s="15" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F76" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G76" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H76" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="23" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>12. RETOURS DU 15/10 (nuit) — habilitations, facturation, échéance</t>
         </is>
       </c>
-      <c r="B78" s="21" t="n"/>
-      <c r="C78" s="21" t="n"/>
-      <c r="D78" s="21" t="n"/>
-      <c r="E78" s="21" t="n"/>
-      <c r="F78" s="21" t="n"/>
-      <c r="G78" s="21" t="n"/>
-      <c r="H78" s="21" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>Personnel</t>
         </is>
       </c>
-      <c r="B79" s="15" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>URGENT — mettre à jour les habilitations</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>Produits et Tiers manquaient à la liste ; sept écrans prennent leur droit (livraisons, B2B, Fiscalité &amp; DGI, stickers, consignations, immobilisations, paramètres) ; personne ne perd un écran (lot 82).</t>
         </is>
       </c>
-      <c r="E79" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F79" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G79" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H79" s="15" t="inlineStr">
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G79" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H79" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="14" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>Paramètres</t>
         </is>
       </c>
-      <c r="B80" s="15" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>12.2</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Section Facturation avec cartes</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Offre, échéance, consommation ; cartes avec avantages : renouveler, passer à une offre supérieure (lot 83).</t>
         </is>
       </c>
-      <c r="E80" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F80" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G80" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H80" s="15" t="inlineStr">
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G80" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H80" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="14" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>Abonnements</t>
         </is>
       </c>
-      <c r="B81" s="15" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>12.3</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>Bloquer l'accès à l'échéance</t>
         </is>
       </c>
-      <c r="D81" s="14" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>Espace visible mais inerte, fenêtre « Abonnement à terme » avec Continuer vers la facturation ; le serveur refuse toute action (lot 83).</t>
         </is>
       </c>
-      <c r="E81" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F81" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G81" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H81" s="15" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G81" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H81" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>Paramétrage</t>
         </is>
       </c>
-      <c r="B82" s="15" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>12.4</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>Métier Poissonnerie</t>
         </is>
       </c>
-      <c r="D82" s="14" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>Nouveau métier du parcours (Commerce) : familles et 22 articles (lot 83).</t>
         </is>
       </c>
-      <c r="E82" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F82" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G82" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H82" s="15" t="inlineStr">
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F82" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G82" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H82" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="14" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B83" s="15" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>12.6</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>« Suivant » du domaine bloquait toute la page</t>
         </is>
       </c>
-      <c r="D83" s="14" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>Le parcours se déroule dans la section (domaine, métiers, modules, rayons) sans soumettre ; appliqué à la création, puis prix et stock (lot 85).</t>
         </is>
       </c>
-      <c r="E83" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F83" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G83" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H83" s="15" t="inlineStr">
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G83" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H83" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>Superadmin</t>
         </is>
       </c>
-      <c r="B84" s="15" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>12.7</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Erreur 500 à la suppression d'une entreprise</t>
         </is>
       </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>Suppression en une transaction, en suivant les dépendances ; « eve disagn » avait perdu ses utilisateurs : relancer la suppression après déploiement (lot 84).</t>
         </is>
       </c>
-      <c r="E84" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F84" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G84" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="H84" s="15" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G84" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H84" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="inlineStr">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12.8</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Habilitations proposées = ce que l'entreprise dispose</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Comptabilité fermée : seule « Trésorerie » est offerte au personnel ; les droits suivent les modules et attributions du moment (lot 86).</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F85" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G85" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Jour 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>Abonnements</t>
         </is>
       </c>
-      <c r="B85" s="15" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>12.5</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>API de paiement</t>
         </is>
       </c>
-      <c r="D85" s="14" t="inlineStr">
-        <is>
-          <t>À brancher dès qu'elle est disponible : elle repoussera l'échéance à la place de DC-Knowing.</t>
-        </is>
-      </c>
-      <c r="E85" s="18" t="inlineStr">
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>En attendant l'API : paiement par référence de transaction, confirmé par le superadmin (lot 89). L'API remplacera la confirmation manuelle.</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>Attendu</t>
         </is>
       </c>
-      <c r="F85" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G85" s="22" t="n"/>
-      <c r="H85" s="15" t="inlineStr">
+      <c r="F86" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>Jour 2</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="20" customHeight="1"/>
-    <row r="94" ht="20" customHeight="1"/>
-    <row r="100" ht="20" customHeight="1"/>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>13. RETOURS DU 16/10 — immobilisations, annulation, paiements, liaisons, sécurité</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Immobilisations</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>N'apparaissent que sur attribution du superadmin</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Menu, écrans et dotations fermés tant que l'attribution n'est pas accordée (lot 87).</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F89" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G89" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Annuler une facture non normalisée, stock réinjecté</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Bouton « Annuler » avec motif : avoir interne total, stock réinjecté, badge « Annulée » ; absent sur une facture normalisée (corrigée par avoir) (lot 87).</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F90" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G90" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Moyens de paiement : pas de numéro de compte, mobile money à part</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Plus aucun numéro de compte dans les listes ; Mobile Money a sa propre liste (journaux 5215-5219) et ne paraît plus sous Banque ; moyens de paiement et codes journaux sont une seule et même chose (lot 88).</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F91" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G91" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Stickers</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>13.4</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Paiement par référence et suivi superadmin</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Opérateur, quantité libre, montant estimé, référence ; En cours / Terminé / Échec avec motif ; badges vert-jaune-rouge ; heure de chaque étape ; priorité au tableau ; compteur selon statut ; « Livrée sur l'espace FNE » retirée (lot 89).</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F92" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G92" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Stickers</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>13.5</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Stock renouvelé : avis à l'entreprise</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Le superadmin saisit stock et solde FNE à la clôture ; l'entreprise reçoit l'avis avec les chiffres, ou « à jour après la première normalisation » (lot 89).</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F93" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G93" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>13.6</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Abonnement et réabonnement par référence</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Après l'inscription comme dans Facturation (sauf pass cadeau) ; Superadmin › Paiements d'abonnement : Confirmer / Activer (lot 89).</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F94" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G94" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Normalisation</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Point de vente non activé : le dire clairement</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>« Le point de vente X n'est pas activé sur votre espace FNE » au lieu de « non reconnu », en normalisation unitaire et par lot (lot 90).</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F95" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G95" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Configuration des comptes : section Articles</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Onglet « Par article » : compte hérité affiché, exception saisissable, recherche (lot 91).</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F96" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G96" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Liaisons</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>13.9</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Comptaflow : créer ou lier un dossier existant</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Choix du dossier Comptaflow (#id — nom), nom affiché après liaison ; chaque côté garde ses accès (lot 92). Comptaflow doit honorer le rattachement.</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F97" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G97" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Liaisons</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13.10</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Exercices à déverser, maintenant ou plus tard</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Cases des exercices au superadmin et, à la demande de l'entreprise, sur sa demande de liaison ; case « déverser maintenant » (lot 92).</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F98" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G98" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13.11</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Mettre l'application hors ligne</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Bouton dans Pannes &amp; assistance ; page « maintenance évolutive, ne vous inquiétez pas » avec téléphone et courriel ; le superadmin garde l'accès (lot 93).</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F99" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G99" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13.12</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>L'application est lente</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>gzip et cache des fichiers statiques, cache des routes effectif, comptages répétés supprimés, vente sans N+1, SMTP borné à 5 s (lot 94). Reste le .env serveur : cache et session en fichier.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F100" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G100" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13.13</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Audit complet et attaques</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Aucune faille critique ; .env, .git, journaux inaccessibles ; HSTS, cookie sécurisé, jeton API haché, OAuth avec state, scripts de debug retirés (lot 94).</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F101" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G101" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13.14</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Caisse paginée pour les grands catalogues</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Afficher 60 articles et chercher le reste : à planifier si le catalogue dépasse quelques centaines d'articles.</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F102" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>13.15</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CSP à nonces, secret externe par entreprise</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Durcissements de moyen terme, sans faille ouverte aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F103" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
     <row r="105" ht="20" customHeight="1"/>
     <row r="112" ht="20" customHeight="1"/>
     <row r="118" ht="20" customHeight="1"/>
@@ -3498,20 +4046,21 @@
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H86"/>
-  <mergeCells count="12">
+  <autoFilter ref="A4:H104"/>
+  <mergeCells count="13">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A67:H67"/>
-    <mergeCell ref="A51:H51"/>
     <mergeCell ref="A78:H78"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A88:H88"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Plans et passation : retours du 16/10 (lots 95 a 105)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1055,24 +1055,54 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>14. RETOURS DU 16/10 (suite) - donnees, UX, supervision</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>105</v>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>13/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>74</v>
-      </c>
-      <c r="D18" t="n">
-        <v>66</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="C19" t="n">
+        <v>89</v>
+      </c>
+      <c r="D19" t="n">
+        <v>79</v>
+      </c>
+      <c r="E19" t="n">
         <v>2</v>
       </c>
-      <c r="F18" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" t="n">
+      <c r="F19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1088,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4038,27 +4068,596 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="20" customHeight="1"/>
-    <row r="112" ht="20" customHeight="1"/>
-    <row r="118" ht="20" customHeight="1"/>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>14. RETOURS DU 16/10 (suite) - donnees, UX, supervision</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Comptaflow</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Montants trop eleves : analyse</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>La liaison ne multiplie rien ; des factures d'essai a 7 milliards gonflaient les totaux. Diagnostic et reprise fournis (lots 95-96).</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F106" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G106" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Facture modifiee : ecritures recalculees</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Modifier une facture contre-passe et repasse ses ecritures ; une facture annulee passe en rouge avec son motif (lots 95, 97).</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F107" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G107" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Tresorerie</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>N'encaisser que le du</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>La caisse enregistrait le montant tendu ; plafonne au du, monnaie rendue exclue. Commande de reprise (lot 96).</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F108" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G108" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Comptabilite</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Remise globale d'achat desequilibrait</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>La remise n'etait pas appliquee aux charges ni a la TVA d'achat : corrige (lot 98).</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F109" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G109" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>14.5</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Rayons des seuls metiers ajoutes</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Ajouter un metier ne remontre que ses rayons ; comptes selon la case Comptabilite (lot 98).</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F110" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G110" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Abonnements</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>14.6</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Sur mesure renouvele par reference</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>L'offre sur mesure se regle par reference, au montant du devis (lot 98).</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F111" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G111" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>14.7</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>URGENT - erreur de lettrage a l'encaissement</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Code de lettrage unique : une vente ne tombe plus en erreur 1062 (lot 99).</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F112" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G112" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>14.8</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Suppression d'entreprise bloquee 5 min</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Corbeille : suppression instantanee, effacement en arriere-plan, restauration 30 j, vider la corbeille (lot 100).</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F113" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G113" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14.9</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Pannes en deux onglets pagines</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Ouvertes / Corrigees, chacune paginee ; message de maintenance modifiable hors ligne (lot 101).</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F114" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G114" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Inscription</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14.10</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Acces immediat + avis d'activation</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Apres la reference de paiement, acces immediat avec compte en cours d'activation (~5 min) (lot 102).</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F115" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G115" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>14.11</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Alertes multi-canal + destinataires</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Courriel multi-destinataires et WhatsApp (relais) pour creation, stickers, paiement, panne, attaque ; destinataires reglables (lot 103).</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F116" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G116" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>14.12</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Maintenance et tracabilite (trafic, IP)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Journal du trafic, KPI, graphe en direct, activite par IP, blocage/deblocage d'IP (lot 104).</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F117" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G117" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>14.13</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Tracabilite par entreprise</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Audit : chaque action, qui, quand, d'ou, par entreprise (lot 105).</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F118" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G118" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Securite</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>14.14</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Contre-attaque demandee</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Refusee : riposter est illegal et frappe des tiers. Defense outillee : hors ligne, blocage d'IP, alertes, signalement hebergeur/CERT.</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F119" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>14.15</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Relais d'envoi WhatsApp</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>A brancher : URL d'un relais (Meta Cloud API, Twilio ou pont) dans Pannes et assistance.</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Attendu</t>
+        </is>
+      </c>
+      <c r="F120" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
     <row r="126"/>
     <row r="127"/>
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H104"/>
-  <mergeCells count="13">
+  <autoFilter ref="A4:H121"/>
+  <mergeCells count="14">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A105:H105"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A88:H88"/>
   </mergeCells>

</xml_diff>

<commit_message>
Plans et passation : lots 108 a 113
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1062,10 +1062,10 @@
         <v>105</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>0</v>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>24/26</t>
         </is>
       </c>
     </row>
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>2</v>
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4859,12 +4859,314 @@
         </is>
       </c>
     </row>
-    <row r="126"/>
-    <row r="127"/>
+    <row r="124">
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>14.19</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Facture affichee des la vente</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>Fenetre facture/ticket apres enregistrement ; impression sans 'Factures vente' (ses propres ventes) (lot 108).</t>
+        </is>
+      </c>
+      <c r="E124" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F124" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G124" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H124" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="inlineStr">
+        <is>
+          <t>Habilitations</t>
+        </is>
+      </c>
+      <c r="B125" s="15" t="inlineStr">
+        <is>
+          <t>14.20</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Annuler sur habilitation</t>
+        </is>
+      </c>
+      <c r="D125" s="14" t="inlineStr">
+        <is>
+          <t>Case 'Annuler une facture vente' ; bouton et route gardes (lot 108).</t>
+        </is>
+      </c>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F125" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G125" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H125" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>14.21</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>URGENT - suppression d'admin interne</t>
+        </is>
+      </c>
+      <c r="D126" s="14" t="inlineStr">
+        <is>
+          <t>Class Auth not found corrige ; seul un compte superadmin se supprime d'ici (lot 109).</t>
+        </is>
+      </c>
+      <c r="E126" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F126" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G126" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H126" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B127" s="15" t="inlineStr">
+        <is>
+          <t>14.22</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Recu en plus gros caracteres</t>
+        </is>
+      </c>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>Police du ticket agrandie (ecran et PDF), certification intacte (lot 110).</t>
+        </is>
+      </c>
+      <c r="E127" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F127" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G127" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H127" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>Habilitations</t>
+        </is>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>14.23</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Volet Stock invisible</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>Matrice fidele aux modules ouverts, encadre 'module non ouvert', commande selflow:diagnostic-acces (lot 110).</t>
+        </is>
+      </c>
+      <c r="E128" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F128" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G128" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H128" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilite</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>14.24</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Soldes de depart clients/fournisseurs</t>
+        </is>
+      </c>
+      <c r="D129" s="14" t="inlineStr">
+        <is>
+          <t>Saisie par tiers, KPI initial/regle/reste, reglement deduit (lot 111).</t>
+        </is>
+      </c>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F129" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G129" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H129" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
+          <t>Ventes/Achats</t>
+        </is>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>14.25</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>KPI des factures</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>Vendu, annule, normalise, non normalise (nombre et montant) (lot 112).</t>
+        </is>
+      </c>
+      <c r="E130" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F130" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G130" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H130" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="inlineStr">
+        <is>
+          <t>14.26</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Switch entreprise (assistance)</t>
+        </is>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>Acceder / se connecter en tant que, bandeau, retour, trace d'audit (lot 113).</t>
+        </is>
+      </c>
+      <c r="E131" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F131" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G131" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H131" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
     <row r="141"/>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H124"/>
+  <autoFilter ref="A4:H132"/>
   <mergeCells count="14">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>

</xml_diff>

<commit_message>
Plans et passation : lots 109 a 121
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$144</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1062,10 +1062,10 @@
         <v>105</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>0</v>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>36/38</t>
         </is>
       </c>
     </row>
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>2</v>
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H131"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5163,10 +5163,465 @@
         </is>
       </c>
     </row>
-    <row r="141"/>
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr">
+        <is>
+          <t>Points de vente</t>
+        </is>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>14.27</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Le site actif commande les saisies</t>
+        </is>
+      </c>
+      <c r="D132" s="14" t="inlineStr">
+        <is>
+          <t>Membre affecte lie a son site ; barre laterale cliquable sans site actif (lot 114).</t>
+        </is>
+      </c>
+      <c r="E132" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F132" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G132" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H132" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="inlineStr">
+        <is>
+          <t>14.28</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Fiche d'entreprise et sites au Switch</t>
+        </is>
+      </c>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>Colonne points de vente, fiche detaillee, diagnostic du stock par site (lot 115).</t>
+        </is>
+      </c>
+      <c r="E133" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F133" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G133" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H133" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>14.29</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Presence des utilisateurs</t>
+        </is>
+      </c>
+      <c r="D134" s="14" t="inlineStr">
+        <is>
+          <t>En ligne / hors ligne et duree de la derniere connexion (lot 116).</t>
+        </is>
+      </c>
+      <c r="E134" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F134" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G134" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H134" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>14.30</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Chaque site voit ses articles</t>
+        </is>
+      </c>
+      <c r="D135" s="14" t="inlineStr">
+        <is>
+          <t>Article reference par site ; caisse, stock, catalogue, alertes filtres (lot 116-117).</t>
+        </is>
+      </c>
+      <c r="E135" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F135" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G135" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H135" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>14.31</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>Voir la derniere facture ; page 403 lisible</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>Sans la liste des ventes, la derniere facture ; acces refuse explique (lot 117).</t>
+        </is>
+      </c>
+      <c r="E136" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F136" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G136" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H136" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="inlineStr">
+        <is>
+          <t>Points de vente</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="inlineStr">
+        <is>
+          <t>14.32</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Prix et numeros par site</t>
+        </is>
+      </c>
+      <c r="D137" s="14" t="inlineStr">
+        <is>
+          <t>Prix propre au site ; numeros VTE-BON-... a partir de 1 par site (lot 118).</t>
+        </is>
+      </c>
+      <c r="E137" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F137" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G137" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H137" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t>Superadmin</t>
+        </is>
+      </c>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>14.33</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>Corbeille immediate ; adresse liberee</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Effacement immediat et rapide ; e-mail libere des la mise en corbeille (lots 118-119).</t>
+        </is>
+      </c>
+      <c r="E138" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F138" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G138" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H138" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilite</t>
+        </is>
+      </c>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>14.34</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Creances sans comptabilite</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Dans la Tresorerie, pour qui a le droit, admin et caissier (lots 119-120).</t>
+        </is>
+      </c>
+      <c r="E139" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F139" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G139" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H139" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>14.35</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>Volet Stock ouvert a qui stocke</t>
+        </is>
+      </c>
+      <c r="D140" s="14" t="inlineStr">
+        <is>
+          <t>Article stockable cree = module Stock ouvert (lot 119).</t>
+        </is>
+      </c>
+      <c r="E140" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F140" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G140" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H140" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="inlineStr">
+        <is>
+          <t>Achats</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>14.36</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>BAPA sur choix explicite</t>
+        </is>
+      </c>
+      <c r="D141" s="14" t="inlineStr">
+        <is>
+          <t>Fournisseur sans NCC n'est plus un BAPA ; normalisation d'achat gardee (lot 120).</t>
+        </is>
+      </c>
+      <c r="E141" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F141" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G141" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H141" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="inlineStr">
+        <is>
+          <t>Tiers</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>14.37</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Creances, soldes et tiers par site</t>
+        </is>
+      </c>
+      <c r="D142" s="14" t="inlineStr">
+        <is>
+          <t>Filtre tous / un site ; clients de la caisse par site (lots 120-121).</t>
+        </is>
+      </c>
+      <c r="E142" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F142" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G142" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H142" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="14" t="inlineStr">
+        <is>
+          <t>Points de vente</t>
+        </is>
+      </c>
+      <c r="B143" s="15" t="inlineStr">
+        <is>
+          <t>14.38</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Choisir son point de vente</t>
+        </is>
+      </c>
+      <c r="D143" s="14" t="inlineStr">
+        <is>
+          <t>Un site : actif d'office ; plusieurs : fenetre de choix, sans blocage (lot 121).</t>
+        </is>
+      </c>
+      <c r="E143" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F143" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G143" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H143" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
     <row r="144"/>
   </sheetData>
-  <autoFilter ref="A4:H132"/>
+  <autoFilter ref="A4:H144"/>
   <mergeCells count="14">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>

</xml_diff>

<commit_message>
Plans et passation : lot 122
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-RETOURS-PRODUCTION.xlsx
+++ b/PLAN-RETOURS-PRODUCTION.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1062,10 +1062,10 @@
         <v>105</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>0</v>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>36/38</t>
+          <t>37/39</t>
         </is>
       </c>
     </row>
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>2</v>
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5619,9 +5619,46 @@
         </is>
       </c>
     </row>
-    <row r="144"/>
+    <row r="144">
+      <c r="A144" s="14" t="inlineStr">
+        <is>
+          <t>Points de vente</t>
+        </is>
+      </c>
+      <c r="B144" s="15" t="inlineStr">
+        <is>
+          <t>14.39</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Doublons de points de vente</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>Cle d'identite, noms proches signales, commande de liste et de fusion (lot 122).</t>
+        </is>
+      </c>
+      <c r="E144" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F144" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G144" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H144" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H144"/>
+  <autoFilter ref="A4:H145"/>
   <mergeCells count="14">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A51:H51"/>

</xml_diff>